<commit_message>
graphen aufgabe 3 E7
</commit_message>
<xml_diff>
--- a/Versuch E7/Daten_E7_Gruppe_8_Kanja_Dagosto.xlsx
+++ b/Versuch E7/Daten_E7_Gruppe_8_Kanja_Dagosto.xlsx
@@ -8,21 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fynnlucca/Documents/Grundpraktikum-1/Versuch E7/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F79DC53-1059-3844-BAD4-41D4F1F12A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D732E5B1-9B5A-2442-9AB3-40C756290EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{FBA0A028-EC3D-6B4A-B90B-9ACFCA4EBE57}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20240" xr2:uid="{FBA0A028-EC3D-6B4A-B90B-9ACFCA4EBE57}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$AQ$7:$AQ$53</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$AR$7:$AR$53</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$AQ$7:$AQ$53</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$AR$7:$AR$53</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$AQ$7:$AQ$53</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$AR$7:$AR$53</definedName>
-  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2299,7 +2291,7 @@
     </row>
     <row r="63" spans="1:56" x14ac:dyDescent="0.2">
       <c r="P63">
-        <v>1480</v>
+        <v>2480</v>
       </c>
       <c r="Q63">
         <v>700</v>

</xml_diff>